<commit_message>
ELV: graficos dos resultados
</commit_message>
<xml_diff>
--- a/data/rebio23-peixes_5-10.xlsx
+++ b/data/rebio23-peixes_5-10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/480d9b848b88e342/MSS/_rebio23-mxr/mxr23_Q/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="933" documentId="11_87A01740D38F142439A96272557A2286C1160297" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7511363-760C-4CEE-87FA-9DBDCBC42F5D}"/>
+  <xr:revisionPtr revIDLastSave="942" documentId="11_87A01740D38F142439A96272557A2286C1160297" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F98FCEA-235E-4318-90FA-38C05C6E7CDB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="637" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10749" uniqueCount="731">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10735" uniqueCount="730">
   <si>
     <t>Etiqueta (C-P-P)</t>
   </si>
@@ -1710,9 +1710,6 @@
     <t>P20</t>
   </si>
   <si>
-    <t>erro</t>
-  </si>
-  <si>
     <t>P54</t>
   </si>
   <si>
@@ -2425,6 +2422,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
@@ -37455,7 +37456,7 @@
         <v>458</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="Q1" s="4" t="s">
         <v>459</v>
@@ -37530,10 +37531,10 @@
         <v>521</v>
       </c>
       <c r="AO1" s="4" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="AP1" s="4" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="AQ1" s="4" t="s">
         <v>522</v>
@@ -37551,13 +37552,13 @@
         <v>526</v>
       </c>
       <c r="AV1" s="4" t="s">
+        <v>724</v>
+      </c>
+      <c r="AW1" s="4" t="s">
         <v>725</v>
       </c>
-      <c r="AW1" s="4" t="s">
+      <c r="AX1" s="4" t="s">
         <v>726</v>
-      </c>
-      <c r="AX1" s="4" t="s">
-        <v>727</v>
       </c>
       <c r="AY1" s="23"/>
       <c r="AZ1" s="23"/>
@@ -37667,7 +37668,10 @@
         <v>68909.705882352951</v>
       </c>
       <c r="AU2" s="23"/>
-      <c r="AW2" s="13"/>
+      <c r="AW2" s="13">
+        <f>COUNTA(AW5:AW677)</f>
+        <v>75</v>
+      </c>
       <c r="AX2" s="23"/>
       <c r="AY2" s="23"/>
       <c r="AZ2" s="23"/>
@@ -38961,7 +38965,7 @@
     </row>
     <row r="15" spans="1:52" ht="12.75" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>481</v>
@@ -39026,10 +39030,10 @@
         <v>540</v>
       </c>
       <c r="W15" s="4" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="X15" s="4" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="Y15" s="27">
         <v>1</v>
@@ -39091,7 +39095,7 @@
     </row>
     <row r="16" spans="1:52" ht="12.75" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B16" s="9" t="s">
         <v>481</v>
@@ -39156,10 +39160,10 @@
         <v>540</v>
       </c>
       <c r="W16" s="4" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="X16" s="4" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="Y16" s="27">
         <v>2</v>
@@ -39221,7 +39225,7 @@
     </row>
     <row r="17" spans="1:50" ht="12.75" customHeight="1">
       <c r="A17" s="4" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>481</v>
@@ -39286,10 +39290,10 @@
         <v>540</v>
       </c>
       <c r="W17" s="4" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="X17" s="4" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="Y17" s="27">
         <v>3</v>
@@ -39351,7 +39355,7 @@
     </row>
     <row r="18" spans="1:50" ht="12.75" customHeight="1">
       <c r="A18" s="4" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B18" s="9" t="s">
         <v>481</v>
@@ -39416,10 +39420,10 @@
         <v>540</v>
       </c>
       <c r="W18" s="4" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="X18" s="4" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="Y18" s="27">
         <v>4</v>
@@ -39481,7 +39485,7 @@
     </row>
     <row r="19" spans="1:50" ht="12.75" customHeight="1">
       <c r="A19" s="4" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>481</v>
@@ -39546,10 +39550,10 @@
         <v>540</v>
       </c>
       <c r="W19" s="4" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="X19" s="4" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="Y19" s="27">
         <v>5</v>
@@ -39611,7 +39615,7 @@
     </row>
     <row r="20" spans="1:50" ht="12.75" customHeight="1">
       <c r="A20" s="4" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B20" s="9" t="s">
         <v>481</v>
@@ -39676,10 +39680,10 @@
         <v>540</v>
       </c>
       <c r="W20" s="4" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="X20" s="4" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="Y20" s="27">
         <v>6</v>
@@ -40068,7 +40072,7 @@
     </row>
     <row r="24" spans="1:50" ht="12.75" customHeight="1">
       <c r="A24" s="4" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B24" s="9" t="s">
         <v>487</v>
@@ -40133,10 +40137,10 @@
         <v>540</v>
       </c>
       <c r="W24" s="4" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="X24" s="4" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="Y24" s="4">
         <v>1</v>
@@ -40179,7 +40183,7 @@
     </row>
     <row r="25" spans="1:50" ht="12.75" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B25" s="9" t="s">
         <v>487</v>
@@ -40244,10 +40248,10 @@
         <v>540</v>
       </c>
       <c r="W25" s="4" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="X25" s="4" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="Y25" s="4">
         <v>2</v>
@@ -40311,7 +40315,7 @@
     </row>
     <row r="26" spans="1:50" ht="12.75" customHeight="1">
       <c r="A26" s="4" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B26" s="9" t="s">
         <v>487</v>
@@ -40376,10 +40380,10 @@
         <v>540</v>
       </c>
       <c r="W26" s="4" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="X26" s="4" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="Y26" s="4">
         <v>3</v>
@@ -42623,7 +42627,7 @@
     </row>
     <row r="47" spans="1:50" ht="12.75" customHeight="1">
       <c r="A47" s="4" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B47" s="9" t="s">
         <v>489</v>
@@ -42688,16 +42692,16 @@
         <v>540</v>
       </c>
       <c r="W47" s="4" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="X47" s="4" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="Y47" s="4">
         <v>1</v>
       </c>
       <c r="Z47" s="4" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="AA47" s="4">
         <v>1</v>
@@ -42757,7 +42761,7 @@
     </row>
     <row r="48" spans="1:50" ht="12.75" customHeight="1">
       <c r="A48" s="4" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B48" s="9" t="s">
         <v>489</v>
@@ -42822,16 +42826,16 @@
         <v>540</v>
       </c>
       <c r="W48" s="4" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="X48" s="4" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="Y48" s="4">
         <v>2</v>
       </c>
       <c r="Z48" s="4" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="AA48" s="4">
         <v>2</v>
@@ -42888,7 +42892,7 @@
     </row>
     <row r="49" spans="1:50" ht="12.75" customHeight="1">
       <c r="A49" s="4" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B49" s="9" t="s">
         <v>489</v>
@@ -42953,16 +42957,16 @@
         <v>540</v>
       </c>
       <c r="W49" s="4" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="X49" s="4" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="Y49" s="4">
         <v>3</v>
       </c>
       <c r="Z49" s="4" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="AA49" s="4">
         <v>3</v>
@@ -43022,7 +43026,7 @@
     </row>
     <row r="50" spans="1:50" ht="12.75" customHeight="1">
       <c r="A50" s="4" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B50" s="9" t="s">
         <v>489</v>
@@ -43087,16 +43091,16 @@
         <v>540</v>
       </c>
       <c r="W50" s="4" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="X50" s="4" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="Y50" s="4">
         <v>4</v>
       </c>
       <c r="Z50" s="4" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="AA50" s="4">
         <v>4</v>
@@ -43108,27 +43112,6 @@
       <c r="AF50" s="24"/>
       <c r="AG50" s="25"/>
       <c r="AH50" s="25"/>
-      <c r="AJ50" s="4" t="s">
-        <v>555</v>
-      </c>
-      <c r="AK50" s="4" t="s">
-        <v>555</v>
-      </c>
-      <c r="AL50" s="4" t="s">
-        <v>555</v>
-      </c>
-      <c r="AM50" s="4" t="s">
-        <v>555</v>
-      </c>
-      <c r="AN50" s="4" t="s">
-        <v>555</v>
-      </c>
-      <c r="AO50" s="4" t="s">
-        <v>555</v>
-      </c>
-      <c r="AP50" s="4" t="s">
-        <v>555</v>
-      </c>
       <c r="AQ50" s="4">
         <v>1.1026</v>
       </c>
@@ -43153,7 +43136,7 @@
     </row>
     <row r="51" spans="1:50" ht="12.75" customHeight="1">
       <c r="A51" s="4" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B51" s="9" t="s">
         <v>489</v>
@@ -43218,16 +43201,16 @@
         <v>540</v>
       </c>
       <c r="W51" s="4" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="X51" s="4" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="Y51" s="4">
         <v>5</v>
       </c>
       <c r="Z51" s="4" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="AA51" s="4">
         <v>5</v>
@@ -43284,7 +43267,7 @@
     </row>
     <row r="52" spans="1:50" ht="12.75" customHeight="1">
       <c r="A52" s="4" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="B52" s="9" t="s">
         <v>489</v>
@@ -43349,16 +43332,16 @@
         <v>540</v>
       </c>
       <c r="W52" s="4" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="X52" s="4" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="Y52" s="4">
         <v>6</v>
       </c>
       <c r="Z52" s="4" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="AA52" s="4">
         <v>6</v>
@@ -43415,7 +43398,7 @@
     </row>
     <row r="53" spans="1:50" ht="12.75" customHeight="1">
       <c r="A53" s="4" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B53" s="9" t="s">
         <v>489</v>
@@ -43480,16 +43463,16 @@
         <v>540</v>
       </c>
       <c r="W53" s="4" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="X53" s="4" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="Y53" s="4">
         <v>7</v>
       </c>
       <c r="Z53" s="4" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="AA53" s="4">
         <v>7</v>
@@ -43546,7 +43529,7 @@
     </row>
     <row r="54" spans="1:50" ht="12.75" customHeight="1">
       <c r="A54" s="4" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B54" s="9" t="s">
         <v>489</v>
@@ -43611,16 +43594,16 @@
         <v>540</v>
       </c>
       <c r="W54" s="4" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="X54" s="4" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="Y54" s="4">
         <v>8</v>
       </c>
       <c r="Z54" s="4" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="AA54" s="4">
         <v>8</v>
@@ -43680,7 +43663,7 @@
     </row>
     <row r="55" spans="1:50" ht="12.75" customHeight="1">
       <c r="A55" s="4" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B55" s="9" t="s">
         <v>489</v>
@@ -43745,16 +43728,16 @@
         <v>540</v>
       </c>
       <c r="W55" s="4" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="X55" s="4" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="Y55" s="4">
         <v>9</v>
       </c>
       <c r="Z55" s="4" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="AA55" s="4">
         <v>9</v>
@@ -44792,7 +44775,7 @@
     </row>
     <row r="65" spans="1:50" ht="12.75" customHeight="1">
       <c r="A65" s="4" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B65" s="9" t="s">
         <v>481</v>
@@ -44857,16 +44840,16 @@
         <v>540</v>
       </c>
       <c r="W65" s="4" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="X65" s="4" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="Y65" s="4">
         <v>1</v>
       </c>
       <c r="Z65" s="4" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="AA65" s="4">
         <v>1</v>
@@ -44926,7 +44909,7 @@
     </row>
     <row r="66" spans="1:50" ht="12.75" customHeight="1">
       <c r="A66" s="4" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B66" s="9" t="s">
         <v>481</v>
@@ -44991,16 +44974,16 @@
         <v>540</v>
       </c>
       <c r="W66" s="4" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="X66" s="4" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="Y66" s="4">
         <v>2</v>
       </c>
       <c r="Z66" s="4" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="AA66" s="4">
         <v>2</v>
@@ -45060,7 +45043,7 @@
     </row>
     <row r="67" spans="1:50" ht="12.75" customHeight="1">
       <c r="A67" s="4" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="B67" s="9" t="s">
         <v>481</v>
@@ -45125,16 +45108,16 @@
         <v>540</v>
       </c>
       <c r="W67" s="4" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="X67" s="4" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="Y67" s="4">
         <v>3</v>
       </c>
       <c r="Z67" s="4" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="AA67" s="4">
         <v>3</v>
@@ -45191,7 +45174,7 @@
     </row>
     <row r="68" spans="1:50" ht="12.75" customHeight="1">
       <c r="A68" s="4" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B68" s="9" t="s">
         <v>481</v>
@@ -45256,16 +45239,16 @@
         <v>540</v>
       </c>
       <c r="W68" s="4" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="X68" s="4" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="Y68" s="4">
         <v>4</v>
       </c>
       <c r="Z68" s="4" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="AA68" s="4">
         <v>4</v>
@@ -45325,7 +45308,7 @@
     </row>
     <row r="69" spans="1:50" ht="12.75" customHeight="1">
       <c r="A69" s="4" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B69" s="9" t="s">
         <v>481</v>
@@ -45390,16 +45373,16 @@
         <v>540</v>
       </c>
       <c r="W69" s="4" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="X69" s="4" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="Y69" s="4">
         <v>5</v>
       </c>
       <c r="Z69" s="4" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="AA69" s="4">
         <v>5</v>
@@ -45459,7 +45442,7 @@
     </row>
     <row r="70" spans="1:50" ht="12.75" customHeight="1">
       <c r="A70" s="4" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B70" s="9" t="s">
         <v>481</v>
@@ -45524,16 +45507,16 @@
         <v>540</v>
       </c>
       <c r="W70" s="4" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="X70" s="4" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="Y70" s="4">
         <v>6</v>
       </c>
       <c r="Z70" s="4" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="AA70" s="4">
         <v>6</v>
@@ -45593,7 +45576,7 @@
     </row>
     <row r="71" spans="1:50" ht="12.75" customHeight="1">
       <c r="A71" s="4" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B71" s="9" t="s">
         <v>481</v>
@@ -45658,16 +45641,16 @@
         <v>540</v>
       </c>
       <c r="W71" s="4" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="X71" s="4" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="Y71" s="4">
         <v>7</v>
       </c>
       <c r="Z71" s="4" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="AA71" s="4">
         <v>7</v>
@@ -45724,7 +45707,7 @@
     </row>
     <row r="72" spans="1:50" ht="12.75" customHeight="1">
       <c r="A72" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B72" s="9" t="s">
         <v>481</v>
@@ -45789,16 +45772,16 @@
         <v>540</v>
       </c>
       <c r="W72" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="X72" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="Y72" s="4">
         <v>8</v>
       </c>
       <c r="Z72" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="AA72" s="4">
         <v>8</v>
@@ -45855,7 +45838,7 @@
     </row>
     <row r="73" spans="1:50" ht="12.75" customHeight="1">
       <c r="A73" s="4" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B73" s="9" t="s">
         <v>481</v>
@@ -45923,16 +45906,16 @@
         <v>540</v>
       </c>
       <c r="W73" s="4" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="X73" s="4" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="Y73" s="4">
         <v>9</v>
       </c>
       <c r="Z73" s="4" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AA73" s="4">
         <v>9</v>
@@ -45989,7 +45972,7 @@
     </row>
     <row r="74" spans="1:50" ht="12.75" customHeight="1">
       <c r="A74" s="4" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B74" s="9" t="s">
         <v>481</v>
@@ -46054,16 +46037,16 @@
         <v>540</v>
       </c>
       <c r="W74" s="4" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="X74" s="4" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="Y74" s="4">
         <v>10</v>
       </c>
       <c r="Z74" s="4" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="AA74" s="4">
         <v>10</v>
@@ -48800,7 +48783,7 @@
     </row>
     <row r="103" spans="1:50" ht="12.75" customHeight="1">
       <c r="A103" s="4" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="B103" s="9" t="s">
         <v>487</v>
@@ -48865,16 +48848,16 @@
         <v>540</v>
       </c>
       <c r="W103" s="4" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="X103" s="4" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="Y103" s="4">
         <v>1</v>
       </c>
       <c r="Z103" s="4" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="AA103" s="4">
         <v>1</v>
@@ -48934,7 +48917,7 @@
     </row>
     <row r="104" spans="1:50" ht="12.75" customHeight="1">
       <c r="A104" s="4" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B104" s="9" t="s">
         <v>487</v>
@@ -48999,16 +48982,16 @@
         <v>540</v>
       </c>
       <c r="W104" s="4" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="X104" s="4" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="Y104" s="4">
         <v>2</v>
       </c>
       <c r="Z104" s="4" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="AA104" s="4">
         <v>2</v>
@@ -49065,7 +49048,7 @@
     </row>
     <row r="105" spans="1:50" ht="12.75" customHeight="1">
       <c r="A105" s="4" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B105" s="9" t="s">
         <v>487</v>
@@ -49130,16 +49113,16 @@
         <v>540</v>
       </c>
       <c r="W105" s="4" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="X105" s="4" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="Y105" s="4">
         <v>3</v>
       </c>
       <c r="Z105" s="4" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="AA105" s="4">
         <v>3</v>
@@ -49196,7 +49179,7 @@
     </row>
     <row r="106" spans="1:50" ht="12.75" customHeight="1">
       <c r="A106" s="4" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B106" s="9" t="s">
         <v>487</v>
@@ -49261,16 +49244,16 @@
         <v>540</v>
       </c>
       <c r="W106" s="4" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="X106" s="4" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="Y106" s="4">
         <v>4</v>
       </c>
       <c r="Z106" s="4" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="AA106" s="4">
         <v>4</v>
@@ -49327,7 +49310,7 @@
     </row>
     <row r="107" spans="1:50" ht="12.75" customHeight="1">
       <c r="A107" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B107" s="9" t="s">
         <v>487</v>
@@ -49392,16 +49375,16 @@
         <v>540</v>
       </c>
       <c r="W107" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="X107" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="Y107" s="4">
         <v>5</v>
       </c>
       <c r="Z107" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="AA107" s="4">
         <v>5</v>
@@ -49458,7 +49441,7 @@
     </row>
     <row r="108" spans="1:50" ht="12.75" customHeight="1">
       <c r="A108" s="4" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B108" s="9" t="s">
         <v>487</v>
@@ -49523,16 +49506,16 @@
         <v>540</v>
       </c>
       <c r="W108" s="4" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="X108" s="4" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="Y108" s="4">
         <v>6</v>
       </c>
       <c r="Z108" s="4" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="AA108" s="4">
         <v>6</v>
@@ -49589,7 +49572,7 @@
     </row>
     <row r="109" spans="1:50" ht="12.75" customHeight="1">
       <c r="A109" s="4" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B109" s="9" t="s">
         <v>487</v>
@@ -49654,16 +49637,16 @@
         <v>540</v>
       </c>
       <c r="W109" s="4" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="X109" s="4" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="Y109" s="4">
         <v>7</v>
       </c>
       <c r="Z109" s="4" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="AA109" s="4">
         <v>7</v>
@@ -49720,7 +49703,7 @@
     </row>
     <row r="110" spans="1:50" ht="12.75" customHeight="1">
       <c r="A110" s="4" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B110" s="9" t="s">
         <v>487</v>
@@ -49785,16 +49768,16 @@
         <v>540</v>
       </c>
       <c r="W110" s="4" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="X110" s="4" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="Y110" s="4">
         <v>8</v>
       </c>
       <c r="Z110" s="4" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="AA110" s="4">
         <v>8</v>
@@ -49851,7 +49834,7 @@
     </row>
     <row r="111" spans="1:50" ht="12.75" customHeight="1">
       <c r="A111" s="4" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="B111" s="9" t="s">
         <v>487</v>
@@ -49916,16 +49899,16 @@
         <v>540</v>
       </c>
       <c r="W111" s="4" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="X111" s="4" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="Y111" s="4">
         <v>9</v>
       </c>
       <c r="Z111" s="4" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="AA111" s="4">
         <v>9</v>
@@ -49982,7 +49965,7 @@
     </row>
     <row r="112" spans="1:50" ht="12.75" customHeight="1">
       <c r="A112" s="4" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B112" s="9" t="s">
         <v>487</v>
@@ -50047,16 +50030,16 @@
         <v>540</v>
       </c>
       <c r="W112" s="4" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="X112" s="4" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="Y112" s="4">
         <v>10</v>
       </c>
       <c r="Z112" s="4" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="AA112" s="4">
         <v>10</v>
@@ -50184,13 +50167,13 @@
         <v>126</v>
       </c>
       <c r="Y113" s="4" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="Z113" s="4" t="s">
         <v>126</v>
       </c>
       <c r="AA113" s="4" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="AB113" s="20">
         <v>0.90920000000000001</v>
@@ -50293,13 +50276,13 @@
         <v>127</v>
       </c>
       <c r="Y114" s="4" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="Z114" s="4" t="s">
         <v>127</v>
       </c>
       <c r="AA114" s="4" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="AB114" s="20">
         <v>0.93049999999999999</v>
@@ -50402,13 +50385,13 @@
         <v>128</v>
       </c>
       <c r="Y115" s="4" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="Z115" s="4" t="s">
         <v>128</v>
       </c>
       <c r="AA115" s="4" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="AB115" s="20">
         <v>0.91569999999999996</v>
@@ -50511,13 +50494,13 @@
         <v>129</v>
       </c>
       <c r="Y116" s="4" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="Z116" s="4" t="s">
         <v>129</v>
       </c>
       <c r="AA116" s="4" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="AB116" s="20">
         <v>1.1178999999999999</v>
@@ -50620,13 +50603,13 @@
         <v>130</v>
       </c>
       <c r="Y117" s="4" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="Z117" s="4" t="s">
         <v>130</v>
       </c>
       <c r="AA117" s="4" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="AB117" s="20">
         <v>0.93369999999999997</v>
@@ -50697,7 +50680,7 @@
         <v>4</v>
       </c>
       <c r="N118" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O118" s="7">
         <v>34</v>
@@ -50729,13 +50712,13 @@
         <v>131</v>
       </c>
       <c r="Y118" s="4" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="Z118" s="4" t="s">
         <v>131</v>
       </c>
       <c r="AA118" s="4" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="AB118" s="20">
         <v>0.91390000000000005</v>
@@ -50838,13 +50821,13 @@
         <v>132</v>
       </c>
       <c r="Y119" s="4" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="Z119" s="4" t="s">
         <v>132</v>
       </c>
       <c r="AA119" s="4" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="AB119" s="20">
         <v>0.92969999999999997</v>
@@ -50915,7 +50898,7 @@
         <v>4</v>
       </c>
       <c r="N120" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O120" s="7">
         <v>32.799999999999997</v>
@@ -50947,13 +50930,13 @@
         <v>133</v>
       </c>
       <c r="Y120" s="4" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="Z120" s="4" t="s">
         <v>133</v>
       </c>
       <c r="AA120" s="4" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="AB120" s="20">
         <v>0.91239999999999999</v>
@@ -51056,13 +51039,13 @@
         <v>134</v>
       </c>
       <c r="Y121" s="4" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="Z121" s="4" t="s">
         <v>134</v>
       </c>
       <c r="AA121" s="4" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="AB121" s="21">
         <v>0.91610000000000003</v>
@@ -51162,13 +51145,13 @@
         <v>135</v>
       </c>
       <c r="Y122" s="4" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="Z122" s="4" t="s">
         <v>135</v>
       </c>
       <c r="AA122" s="4" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="AB122" s="20">
         <v>0.91559999999999997</v>
@@ -51271,13 +51254,13 @@
         <v>136</v>
       </c>
       <c r="Y123" s="4" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="Z123" s="4" t="s">
         <v>136</v>
       </c>
       <c r="AA123" s="4" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="AB123" s="20">
         <v>0.93010000000000004</v>
@@ -51380,13 +51363,13 @@
         <v>137</v>
       </c>
       <c r="Y124" s="4" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="Z124" s="4" t="s">
         <v>137</v>
       </c>
       <c r="AA124" s="4" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="AB124" s="21">
         <v>0.9204</v>
@@ -51486,13 +51469,13 @@
         <v>138</v>
       </c>
       <c r="Y125" s="4" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="Z125" s="4" t="s">
         <v>138</v>
       </c>
       <c r="AA125" s="4" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="AB125" s="20">
         <v>1.1163000000000001</v>
@@ -51563,7 +51546,7 @@
         <v>4</v>
       </c>
       <c r="N126" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O126" s="7">
         <v>27</v>
@@ -51598,13 +51581,13 @@
         <v>139</v>
       </c>
       <c r="Y126" s="4" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="Z126" s="4" t="s">
         <v>139</v>
       </c>
       <c r="AA126" s="4" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="AB126" s="20">
         <v>1.1226</v>
@@ -51707,13 +51690,13 @@
         <v>143</v>
       </c>
       <c r="Y127" s="4" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="Z127" s="4" t="s">
         <v>143</v>
       </c>
       <c r="AA127" s="4" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="AB127" s="20">
         <v>0.90049999999999997</v>
@@ -51784,7 +51767,7 @@
         <v>4</v>
       </c>
       <c r="N128" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O128" s="7">
         <v>28.5</v>
@@ -51816,13 +51799,13 @@
         <v>144</v>
       </c>
       <c r="Y128" s="4" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="Z128" s="4" t="s">
         <v>144</v>
       </c>
       <c r="AA128" s="4" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="AB128" s="20">
         <v>0.92400000000000004</v>
@@ -51893,7 +51876,7 @@
         <v>4</v>
       </c>
       <c r="N129" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O129" s="4">
         <v>29.6</v>
@@ -51971,7 +51954,7 @@
         <v>4</v>
       </c>
       <c r="N130" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O130" s="4">
         <v>22.2</v>
@@ -52205,7 +52188,7 @@
         <v>4</v>
       </c>
       <c r="N133" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O133" s="4">
         <v>23.8</v>
@@ -52673,7 +52656,7 @@
         <v>4</v>
       </c>
       <c r="N139" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O139" s="4">
         <v>33.6</v>
@@ -52829,7 +52812,7 @@
         <v>4</v>
       </c>
       <c r="N141" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O141" s="4">
         <v>25.2</v>
@@ -53219,7 +53202,7 @@
         <v>4</v>
       </c>
       <c r="N146" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O146" s="4">
         <v>22.1</v>
@@ -53297,7 +53280,7 @@
         <v>4</v>
       </c>
       <c r="N147" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O147" s="4">
         <v>22.4</v>
@@ -53921,7 +53904,7 @@
         <v>4</v>
       </c>
       <c r="N155" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O155" s="4">
         <v>22.2</v>
@@ -54314,7 +54297,7 @@
         <v>4</v>
       </c>
       <c r="N160" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O160" s="4">
         <v>31.2</v>
@@ -54548,7 +54531,7 @@
         <v>4</v>
       </c>
       <c r="N163" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O163" s="4">
         <v>23.5</v>
@@ -55250,7 +55233,7 @@
         <v>4</v>
       </c>
       <c r="N172" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O172" s="4">
         <v>17.3</v>
@@ -55757,7 +55740,7 @@
     </row>
     <row r="179" spans="1:50" ht="12.75" customHeight="1">
       <c r="A179" s="4" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B179" s="9" t="s">
         <v>491</v>
@@ -55822,16 +55805,16 @@
         <v>540</v>
       </c>
       <c r="W179" s="4" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="X179" s="4" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="Y179" s="4">
         <v>1</v>
       </c>
       <c r="Z179" s="4" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="AA179" s="4">
         <v>1</v>
@@ -55888,7 +55871,7 @@
     </row>
     <row r="180" spans="1:50" ht="12.75" customHeight="1">
       <c r="A180" s="4" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B180" s="9" t="s">
         <v>491</v>
@@ -55953,16 +55936,16 @@
         <v>540</v>
       </c>
       <c r="W180" s="4" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="X180" s="4" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="Y180" s="4">
         <v>2</v>
       </c>
       <c r="Z180" s="4" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="AA180" s="4">
         <v>2</v>
@@ -56022,7 +56005,7 @@
     </row>
     <row r="181" spans="1:50" ht="12.75" customHeight="1">
       <c r="A181" s="4" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="B181" s="9" t="s">
         <v>491</v>
@@ -56087,16 +56070,16 @@
         <v>540</v>
       </c>
       <c r="W181" s="4" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="X181" s="4" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="Y181" s="4">
         <v>3</v>
       </c>
       <c r="Z181" s="4" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="AA181" s="4">
         <v>3</v>
@@ -56156,7 +56139,7 @@
     </row>
     <row r="182" spans="1:50" ht="12.75" customHeight="1">
       <c r="A182" s="4" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B182" s="9" t="s">
         <v>491</v>
@@ -56221,16 +56204,16 @@
         <v>540</v>
       </c>
       <c r="W182" s="4" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="X182" s="4" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="Y182" s="4">
         <v>4</v>
       </c>
       <c r="Z182" s="4" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="AA182" s="4">
         <v>4</v>
@@ -56290,7 +56273,7 @@
     </row>
     <row r="183" spans="1:50" ht="12.75" customHeight="1">
       <c r="A183" s="4" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="B183" s="9" t="s">
         <v>491</v>
@@ -56355,16 +56338,16 @@
         <v>540</v>
       </c>
       <c r="W183" s="4" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="X183" s="4" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="Y183" s="4">
         <v>5</v>
       </c>
       <c r="Z183" s="4" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="AA183" s="4">
         <v>5</v>
@@ -56424,7 +56407,7 @@
     </row>
     <row r="184" spans="1:50" ht="12.75" customHeight="1">
       <c r="A184" s="4" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="B184" s="9" t="s">
         <v>491</v>
@@ -56489,16 +56472,16 @@
         <v>540</v>
       </c>
       <c r="W184" s="4" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="X184" s="4" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="Y184" s="4">
         <v>6</v>
       </c>
       <c r="Z184" s="4" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="AA184" s="4">
         <v>6</v>
@@ -56555,7 +56538,7 @@
     </row>
     <row r="185" spans="1:50" ht="12.75" customHeight="1">
       <c r="A185" s="4" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="B185" s="9" t="s">
         <v>491</v>
@@ -56620,16 +56603,16 @@
         <v>540</v>
       </c>
       <c r="W185" s="4" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="X185" s="4" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="Y185" s="4">
         <v>7</v>
       </c>
       <c r="Z185" s="4" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="AA185" s="4">
         <v>7</v>
@@ -56689,7 +56672,7 @@
     </row>
     <row r="186" spans="1:50" ht="12.75" customHeight="1">
       <c r="A186" s="4" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="B186" s="9" t="s">
         <v>491</v>
@@ -56754,16 +56737,16 @@
         <v>540</v>
       </c>
       <c r="W186" s="4" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="X186" s="4" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="Y186" s="4">
         <v>8</v>
       </c>
       <c r="Z186" s="4" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="AA186" s="4">
         <v>8</v>
@@ -56823,7 +56806,7 @@
     </row>
     <row r="187" spans="1:50" ht="12.75" customHeight="1">
       <c r="A187" s="4" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="B187" s="9" t="s">
         <v>491</v>
@@ -56888,16 +56871,16 @@
         <v>540</v>
       </c>
       <c r="W187" s="4" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="X187" s="4" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="Y187" s="4">
         <v>9</v>
       </c>
       <c r="Z187" s="4" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="AA187" s="4">
         <v>9</v>
@@ -56954,7 +56937,7 @@
     </row>
     <row r="188" spans="1:50" ht="12.75" customHeight="1">
       <c r="A188" s="4" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="B188" s="9" t="s">
         <v>491</v>
@@ -56993,7 +56976,7 @@
         <v>4</v>
       </c>
       <c r="N188" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O188" s="7">
         <v>34.299999999999997</v>
@@ -57019,16 +57002,16 @@
         <v>540</v>
       </c>
       <c r="W188" s="4" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="X188" s="4" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="Y188" s="4">
         <v>10</v>
       </c>
       <c r="Z188" s="4" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="AA188" s="4">
         <v>10</v>
@@ -57088,7 +57071,7 @@
     </row>
     <row r="189" spans="1:50" ht="12.75" customHeight="1">
       <c r="A189" s="4" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="B189" s="9" t="s">
         <v>491</v>
@@ -57153,16 +57136,16 @@
         <v>540</v>
       </c>
       <c r="W189" s="4" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="X189" s="4" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="Y189" s="4">
         <v>11</v>
       </c>
       <c r="Z189" s="4" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="AA189" s="4">
         <v>11</v>
@@ -57222,7 +57205,7 @@
     </row>
     <row r="190" spans="1:50" ht="12.75" customHeight="1">
       <c r="A190" s="4" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="B190" s="9" t="s">
         <v>491</v>
@@ -57287,16 +57270,16 @@
         <v>540</v>
       </c>
       <c r="W190" s="4" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="X190" s="4" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="Y190" s="4">
         <v>12</v>
       </c>
       <c r="Z190" s="4" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="AA190" s="4">
         <v>12</v>
@@ -57356,7 +57339,7 @@
     </row>
     <row r="191" spans="1:50" ht="12.75" customHeight="1">
       <c r="A191" s="4" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="B191" s="9" t="s">
         <v>491</v>
@@ -57421,16 +57404,16 @@
         <v>540</v>
       </c>
       <c r="W191" s="4" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="X191" s="4" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="Y191" s="4">
         <v>13</v>
       </c>
       <c r="Z191" s="4" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="AA191" s="4">
         <v>13</v>
@@ -57487,7 +57470,7 @@
     </row>
     <row r="192" spans="1:50" ht="12.75" customHeight="1">
       <c r="A192" s="4" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="B192" s="14" t="s">
         <v>491</v>
@@ -57526,7 +57509,7 @@
         <v>4</v>
       </c>
       <c r="N192" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O192" s="4">
         <v>28.6</v>
@@ -57552,7 +57535,7 @@
         <v>533</v>
       </c>
       <c r="W192" s="4" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="AB192" s="20"/>
       <c r="AC192" s="20"/>
@@ -57604,7 +57587,7 @@
         <v>3</v>
       </c>
       <c r="N193" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O193" s="7">
         <v>24.8</v>
@@ -57636,13 +57619,13 @@
         <v>212</v>
       </c>
       <c r="Y193" s="4" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="Z193" s="4" t="s">
         <v>212</v>
       </c>
       <c r="AA193" s="4" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="AB193" s="20">
         <v>1.1154999999999999</v>
@@ -57745,13 +57728,13 @@
         <v>213</v>
       </c>
       <c r="Y194" s="4" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="Z194" s="4" t="s">
         <v>213</v>
       </c>
       <c r="AA194" s="4" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="AB194" s="20">
         <v>0.93559999999999999</v>
@@ -57854,13 +57837,13 @@
         <v>214</v>
       </c>
       <c r="Y195" s="4" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="Z195" s="4" t="s">
         <v>214</v>
       </c>
       <c r="AA195" s="4" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="AB195" s="20">
         <v>0.90369999999999995</v>
@@ -57963,13 +57946,13 @@
         <v>215</v>
       </c>
       <c r="Y196" s="4" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="Z196" s="4" t="s">
         <v>215</v>
       </c>
       <c r="AA196" s="4" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="AB196" s="20">
         <v>0.91459999999999997</v>
@@ -58072,13 +58055,13 @@
         <v>216</v>
       </c>
       <c r="Y197" s="4" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="Z197" s="4" t="s">
         <v>216</v>
       </c>
       <c r="AA197" s="4" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="AB197" s="20">
         <v>1.1163000000000001</v>
@@ -58181,13 +58164,13 @@
         <v>217</v>
       </c>
       <c r="Y198" s="4" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="Z198" s="4" t="s">
         <v>217</v>
       </c>
       <c r="AA198" s="4" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AB198" s="20">
         <v>0.91739999999999999</v>
@@ -58290,13 +58273,13 @@
         <v>218</v>
       </c>
       <c r="Y199" s="4" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="Z199" s="4" t="s">
         <v>218</v>
       </c>
       <c r="AA199" s="4" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AB199" s="20">
         <v>1.1106</v>
@@ -58399,13 +58382,13 @@
         <v>219</v>
       </c>
       <c r="Y200" s="4" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="Z200" s="4" t="s">
         <v>219</v>
       </c>
       <c r="AA200" s="4" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="AB200" s="20">
         <v>0.89959999999999996</v>
@@ -58508,13 +58491,13 @@
         <v>220</v>
       </c>
       <c r="Y201" s="4" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="Z201" s="4" t="s">
         <v>220</v>
       </c>
       <c r="AA201" s="4" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AB201" s="20">
         <v>0.91310000000000002</v>
@@ -58617,13 +58600,13 @@
         <v>221</v>
       </c>
       <c r="Y202" s="4" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="Z202" s="4" t="s">
         <v>221</v>
       </c>
       <c r="AA202" s="4" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AB202" s="20">
         <v>1.1022000000000001</v>
@@ -58726,13 +58709,13 @@
         <v>222</v>
       </c>
       <c r="Y203" s="4" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="Z203" s="4" t="s">
         <v>222</v>
       </c>
       <c r="AA203" s="4" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="AB203" s="20">
         <v>1.1003000000000001</v>
@@ -58835,13 +58818,13 @@
         <v>223</v>
       </c>
       <c r="Y204" s="4" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="Z204" s="4" t="s">
         <v>223</v>
       </c>
       <c r="AA204" s="4" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="AB204" s="20">
         <v>0.93400000000000005</v>
@@ -58944,13 +58927,13 @@
         <v>224</v>
       </c>
       <c r="Y205" s="4" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="Z205" s="4" t="s">
         <v>224</v>
       </c>
       <c r="AA205" s="4" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="AB205" s="20">
         <v>0.91959999999999997</v>
@@ -59053,13 +59036,13 @@
         <v>225</v>
       </c>
       <c r="Y206" s="4" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="Z206" s="4" t="s">
         <v>225</v>
       </c>
       <c r="AA206" s="4" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="AB206" s="20">
         <v>0.93269999999999997</v>
@@ -59162,13 +59145,13 @@
         <v>226</v>
       </c>
       <c r="Y207" s="4" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="Z207" s="4" t="s">
         <v>226</v>
       </c>
       <c r="AA207" s="4" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AB207" s="20">
         <v>0.92949999999999999</v>
@@ -59229,11 +59212,11 @@
       <c r="W208" s="7"/>
       <c r="X208" s="7"/>
       <c r="Y208" s="4" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="Z208" s="7"/>
       <c r="AA208" s="4" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="AB208" s="21">
         <v>0.92500000000000004</v>
@@ -59319,13 +59302,13 @@
         <v>227</v>
       </c>
       <c r="Y209" s="4" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="Z209" s="4" t="s">
         <v>227</v>
       </c>
       <c r="AA209" s="4" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="AB209" s="20">
         <v>0.93279999999999996</v>
@@ -59396,7 +59379,7 @@
         <v>3</v>
       </c>
       <c r="N210" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O210" s="7">
         <v>27.5</v>
@@ -59428,13 +59411,13 @@
         <v>228</v>
       </c>
       <c r="Y210" s="4" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="Z210" s="4" t="s">
         <v>228</v>
       </c>
       <c r="AA210" s="4" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="AB210" s="20">
         <v>1.1354</v>
@@ -59537,13 +59520,13 @@
         <v>229</v>
       </c>
       <c r="Y211" s="4" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="Z211" s="4" t="s">
         <v>229</v>
       </c>
       <c r="AA211" s="4" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="AB211" s="20">
         <v>1.1025</v>
@@ -59646,13 +59629,13 @@
         <v>231</v>
       </c>
       <c r="Y212" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="Z212" s="4" t="s">
         <v>231</v>
       </c>
       <c r="AA212" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="AB212" s="20">
         <v>0.93130000000000002</v>
@@ -59755,13 +59738,13 @@
         <v>232</v>
       </c>
       <c r="Y213" s="4" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="Z213" s="4" t="s">
         <v>232</v>
       </c>
       <c r="AA213" s="4" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="AB213" s="20">
         <v>0.93049999999999999</v>
@@ -59864,13 +59847,13 @@
         <v>233</v>
       </c>
       <c r="Y214" s="4" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="Z214" s="4" t="s">
         <v>233</v>
       </c>
       <c r="AA214" s="4" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="AB214" s="20">
         <v>0.91539999999999999</v>
@@ -60409,7 +60392,7 @@
         <v>3</v>
       </c>
       <c r="N221" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O221" s="4">
         <v>27.8</v>
@@ -60565,7 +60548,7 @@
         <v>3</v>
       </c>
       <c r="N223" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O223" s="4">
         <v>29.1</v>
@@ -61501,7 +61484,7 @@
         <v>3</v>
       </c>
       <c r="N235" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O235" s="4">
         <v>30.9</v>
@@ -65248,7 +65231,7 @@
         <v>3</v>
       </c>
       <c r="N283" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O283" s="4">
         <v>29.9</v>
@@ -65878,7 +65861,7 @@
         <v>3</v>
       </c>
       <c r="N291" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O291" s="4">
         <v>23.8</v>
@@ -66034,7 +66017,7 @@
         <v>3</v>
       </c>
       <c r="N293" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O293" s="4">
         <v>22.2</v>
@@ -66544,7 +66527,7 @@
     </row>
     <row r="300" spans="1:50">
       <c r="A300" s="4" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="B300" s="9" t="s">
         <v>494</v>
@@ -66609,16 +66592,16 @@
         <v>540</v>
       </c>
       <c r="W300" s="4" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="X300" s="4" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="Y300" s="4">
         <v>1</v>
       </c>
       <c r="Z300" s="4" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="AA300" s="4">
         <v>1</v>
@@ -66678,7 +66661,7 @@
     </row>
     <row r="301" spans="1:50">
       <c r="A301" s="4" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="B301" s="9" t="s">
         <v>494</v>
@@ -66743,16 +66726,16 @@
         <v>540</v>
       </c>
       <c r="W301" s="4" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="X301" s="4" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="Y301" s="4">
         <v>2</v>
       </c>
       <c r="Z301" s="4" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="AA301" s="4">
         <v>2</v>
@@ -66812,7 +66795,7 @@
     </row>
     <row r="302" spans="1:50">
       <c r="A302" s="4" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="B302" s="9" t="s">
         <v>494</v>
@@ -66877,16 +66860,16 @@
         <v>540</v>
       </c>
       <c r="W302" s="4" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="X302" s="4" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="Y302" s="4">
         <v>3</v>
       </c>
       <c r="Z302" s="4" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="AA302" s="4">
         <v>3</v>
@@ -66946,7 +66929,7 @@
     </row>
     <row r="303" spans="1:50">
       <c r="A303" s="4" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B303" s="9" t="s">
         <v>494</v>
@@ -67011,16 +66994,16 @@
         <v>540</v>
       </c>
       <c r="W303" s="4" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="X303" s="4" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="Y303" s="4">
         <v>4</v>
       </c>
       <c r="Z303" s="4" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="AA303" s="4">
         <v>4</v>
@@ -67080,7 +67063,7 @@
     </row>
     <row r="304" spans="1:50">
       <c r="A304" s="4" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="B304" s="9" t="s">
         <v>494</v>
@@ -67145,16 +67128,16 @@
         <v>540</v>
       </c>
       <c r="W304" s="4" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="X304" s="4" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="Y304" s="4">
         <v>5</v>
       </c>
       <c r="Z304" s="4" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="AA304" s="4">
         <v>5</v>
@@ -67214,7 +67197,7 @@
     </row>
     <row r="305" spans="1:50">
       <c r="A305" s="4" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="B305" s="9" t="s">
         <v>494</v>
@@ -67279,16 +67262,16 @@
         <v>540</v>
       </c>
       <c r="W305" s="4" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="X305" s="4" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="Y305" s="4">
         <v>6</v>
       </c>
       <c r="Z305" s="4" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="AA305" s="4">
         <v>6</v>
@@ -67348,7 +67331,7 @@
     </row>
     <row r="306" spans="1:50">
       <c r="A306" s="4" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="B306" s="9" t="s">
         <v>494</v>
@@ -67413,16 +67396,16 @@
         <v>540</v>
       </c>
       <c r="W306" s="4" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="X306" s="4" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="Y306" s="4">
         <v>7</v>
       </c>
       <c r="Z306" s="4" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="AA306" s="4">
         <v>7</v>
@@ -67482,7 +67465,7 @@
     </row>
     <row r="307" spans="1:50">
       <c r="A307" s="4" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="B307" s="9" t="s">
         <v>494</v>
@@ -67547,16 +67530,16 @@
         <v>540</v>
       </c>
       <c r="W307" s="4" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="X307" s="4" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="Y307" s="4">
         <v>8</v>
       </c>
       <c r="Z307" s="4" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="AA307" s="4">
         <v>8</v>
@@ -67616,7 +67599,7 @@
     </row>
     <row r="308" spans="1:50">
       <c r="A308" s="4" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="B308" s="9" t="s">
         <v>494</v>
@@ -67681,16 +67664,16 @@
         <v>540</v>
       </c>
       <c r="W308" s="4" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="X308" s="4" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="Y308" s="4">
         <v>9</v>
       </c>
       <c r="Z308" s="4" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="AA308" s="4">
         <v>9</v>
@@ -67747,7 +67730,7 @@
     </row>
     <row r="309" spans="1:50">
       <c r="A309" s="4" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="B309" s="9" t="s">
         <v>494</v>
@@ -67812,16 +67795,16 @@
         <v>540</v>
       </c>
       <c r="W309" s="4" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="X309" s="4" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="Y309" s="4">
         <v>10</v>
       </c>
       <c r="Z309" s="4" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="AA309" s="4">
         <v>10</v>
@@ -67878,7 +67861,7 @@
     </row>
     <row r="310" spans="1:50">
       <c r="A310" s="4" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="B310" s="9" t="s">
         <v>494</v>
@@ -67943,16 +67926,16 @@
         <v>540</v>
       </c>
       <c r="W310" s="4" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="X310" s="4" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="Y310" s="4">
         <v>11</v>
       </c>
       <c r="Z310" s="4" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="AA310" s="4">
         <v>11</v>
@@ -68012,7 +67995,7 @@
     </row>
     <row r="311" spans="1:50">
       <c r="A311" s="4" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="B311" s="9" t="s">
         <v>494</v>
@@ -68077,16 +68060,16 @@
         <v>540</v>
       </c>
       <c r="W311" s="4" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="X311" s="4" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="Y311" s="4">
         <v>12</v>
       </c>
       <c r="Z311" s="4" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="AA311" s="4">
         <v>12</v>
@@ -68146,7 +68129,7 @@
     </row>
     <row r="312" spans="1:50">
       <c r="A312" s="4" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="B312" s="9" t="s">
         <v>494</v>
@@ -68211,16 +68194,16 @@
         <v>540</v>
       </c>
       <c r="W312" s="4" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="X312" s="4" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="Y312" s="4">
         <v>13</v>
       </c>
       <c r="Z312" s="4" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="AA312" s="4">
         <v>13</v>
@@ -68280,7 +68263,7 @@
     </row>
     <row r="313" spans="1:50">
       <c r="A313" s="28" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="B313" s="29" t="s">
         <v>491</v>
@@ -68319,7 +68302,7 @@
         <v>4</v>
       </c>
       <c r="N313" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O313" s="7">
         <v>34.799999999999997</v>
@@ -68348,16 +68331,16 @@
         <v>540</v>
       </c>
       <c r="W313" s="4" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="X313" s="4" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="Y313" s="4">
         <v>14</v>
       </c>
       <c r="Z313" s="4" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="AA313" s="4">
         <v>14</v>
@@ -68417,7 +68400,7 @@
     </row>
     <row r="314" spans="1:50">
       <c r="A314" s="4" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="B314" s="9" t="s">
         <v>494</v>
@@ -68482,16 +68465,16 @@
         <v>540</v>
       </c>
       <c r="W314" s="4" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="X314" s="4" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="Y314" s="4">
         <v>14</v>
       </c>
       <c r="Z314" s="4" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="AA314" s="4">
         <v>14</v>
@@ -68548,7 +68531,7 @@
     </row>
     <row r="315" spans="1:50" ht="12.75" customHeight="1">
       <c r="A315" s="4" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="B315" s="14" t="s">
         <v>494</v>
@@ -68613,7 +68596,7 @@
         <v>533</v>
       </c>
       <c r="W315" s="4" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="AB315" s="20"/>
       <c r="AC315" s="20"/>
@@ -68626,7 +68609,7 @@
     </row>
     <row r="316" spans="1:50" ht="12.75" customHeight="1">
       <c r="A316" s="4" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="B316" s="14" t="s">
         <v>494</v>
@@ -68691,7 +68674,7 @@
         <v>533</v>
       </c>
       <c r="W316" s="4" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="AB316" s="20"/>
       <c r="AC316" s="20"/>
@@ -68704,7 +68687,7 @@
     </row>
     <row r="317" spans="1:50" ht="12.75" customHeight="1">
       <c r="A317" s="4" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="B317" s="14" t="s">
         <v>494</v>
@@ -68743,7 +68726,7 @@
         <v>3</v>
       </c>
       <c r="N317" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O317" s="4">
         <v>16.600000000000001</v>
@@ -68769,7 +68752,7 @@
         <v>533</v>
       </c>
       <c r="W317" s="4" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="AB317" s="20"/>
       <c r="AC317" s="20"/>
@@ -68853,13 +68836,13 @@
         <v>347</v>
       </c>
       <c r="Y318" s="4" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="Z318" s="4" t="s">
         <v>347</v>
       </c>
       <c r="AA318" s="4" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="AB318" s="20">
         <v>0.92349999999999999</v>
@@ -68962,13 +68945,13 @@
         <v>348</v>
       </c>
       <c r="Y319" s="4" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="Z319" s="4" t="s">
         <v>348</v>
       </c>
       <c r="AA319" s="4" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="AB319" s="20">
         <v>0.90069999999999995</v>
@@ -69071,13 +69054,13 @@
         <v>349</v>
       </c>
       <c r="Y320" s="4" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="Z320" s="4" t="s">
         <v>349</v>
       </c>
       <c r="AA320" s="4" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="AB320" s="20">
         <v>1.1238999999999999</v>
@@ -69180,13 +69163,13 @@
         <v>350</v>
       </c>
       <c r="Y321" s="4" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="Z321" s="4" t="s">
         <v>350</v>
       </c>
       <c r="AA321" s="4" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="AB321" s="20">
         <v>1.1348</v>
@@ -69257,7 +69240,7 @@
         <v>4</v>
       </c>
       <c r="N322" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O322" s="7">
         <v>28.6</v>
@@ -69289,13 +69272,13 @@
         <v>351</v>
       </c>
       <c r="Y322" s="4" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="Z322" s="4" t="s">
         <v>351</v>
       </c>
       <c r="AA322" s="4" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="AB322" s="20">
         <v>0.93379999999999996</v>
@@ -69398,13 +69381,13 @@
         <v>352</v>
       </c>
       <c r="Y323" s="4" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="Z323" s="4" t="s">
         <v>352</v>
       </c>
       <c r="AA323" s="4" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="AB323" s="20">
         <v>0.91810000000000003</v>
@@ -69475,7 +69458,7 @@
         <v>4</v>
       </c>
       <c r="N324" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O324" s="7">
         <v>30.1</v>
@@ -69507,13 +69490,13 @@
         <v>353</v>
       </c>
       <c r="Y324" s="4" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="Z324" s="4" t="s">
         <v>353</v>
       </c>
       <c r="AA324" s="4" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="AB324" s="20">
         <v>0.91720000000000002</v>
@@ -69616,13 +69599,13 @@
         <v>354</v>
       </c>
       <c r="Y325" s="4" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="Z325" s="4" t="s">
         <v>354</v>
       </c>
       <c r="AA325" s="4" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="AB325" s="20">
         <v>1.0974999999999999</v>
@@ -69693,7 +69676,7 @@
         <v>4</v>
       </c>
       <c r="N326" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O326" s="7">
         <v>29.4</v>
@@ -69725,13 +69708,13 @@
         <v>355</v>
       </c>
       <c r="Y326" s="4" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="Z326" s="4" t="s">
         <v>355</v>
       </c>
       <c r="AA326" s="4" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="AB326" s="20">
         <v>0.90910000000000002</v>
@@ -69834,13 +69817,13 @@
         <v>356</v>
       </c>
       <c r="Y327" s="4" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="Z327" s="4" t="s">
         <v>356</v>
       </c>
       <c r="AA327" s="4" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="AB327" s="20">
         <v>0.9123</v>
@@ -69911,7 +69894,7 @@
         <v>4</v>
       </c>
       <c r="N328" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O328" s="7">
         <v>14.7</v>
@@ -69943,13 +69926,13 @@
         <v>357</v>
       </c>
       <c r="Y328" s="4" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="Z328" s="4" t="s">
         <v>357</v>
       </c>
       <c r="AA328" s="4" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="AB328" s="20">
         <v>0.90910000000000002</v>
@@ -70052,13 +70035,13 @@
         <v>358</v>
       </c>
       <c r="Y329" s="4" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="Z329" s="4" t="s">
         <v>358</v>
       </c>
       <c r="AA329" s="4" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="AB329" s="20">
         <v>0.92290000000000005</v>
@@ -70129,7 +70112,7 @@
         <v>4</v>
       </c>
       <c r="N330" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O330" s="7">
         <v>28</v>
@@ -70161,13 +70144,13 @@
         <v>359</v>
       </c>
       <c r="Y330" s="4" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="Z330" s="4" t="s">
         <v>359</v>
       </c>
       <c r="AA330" s="4" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="AB330" s="20">
         <v>0.90849999999999997</v>
@@ -70270,13 +70253,13 @@
         <v>360</v>
       </c>
       <c r="Y331" s="4" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="Z331" s="4" t="s">
         <v>360</v>
       </c>
       <c r="AA331" s="4" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="AB331" s="20">
         <v>0.93069999999999997</v>
@@ -70379,13 +70362,13 @@
         <v>361</v>
       </c>
       <c r="Y332" s="4" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="Z332" s="4" t="s">
         <v>361</v>
       </c>
       <c r="AA332" s="4" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="AB332" s="20">
         <v>0.9284</v>
@@ -70456,7 +70439,7 @@
         <v>4</v>
       </c>
       <c r="N333" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O333" s="7">
         <v>25.8</v>
@@ -70488,13 +70471,13 @@
         <v>362</v>
       </c>
       <c r="Y333" s="4" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="Z333" s="4" t="s">
         <v>362</v>
       </c>
       <c r="AA333" s="4" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="AB333" s="20">
         <v>0.93520000000000003</v>
@@ -70597,13 +70580,13 @@
         <v>363</v>
       </c>
       <c r="Y334" s="4" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="Z334" s="4" t="s">
         <v>363</v>
       </c>
       <c r="AA334" s="4" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="AB334" s="20">
         <v>0.93240000000000001</v>
@@ -70706,13 +70689,13 @@
         <v>364</v>
       </c>
       <c r="Y335" s="4" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="Z335" s="4" t="s">
         <v>364</v>
       </c>
       <c r="AA335" s="4" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="AB335" s="20">
         <v>0.92210000000000003</v>
@@ -70815,13 +70798,13 @@
         <v>365</v>
       </c>
       <c r="Y336" s="4" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="Z336" s="4" t="s">
         <v>365</v>
       </c>
       <c r="AA336" s="4" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="AB336" s="20">
         <v>1.1026</v>
@@ -70892,7 +70875,7 @@
         <v>4</v>
       </c>
       <c r="N337" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O337" s="7">
         <v>34.700000000000003</v>
@@ -70924,13 +70907,13 @@
         <v>366</v>
       </c>
       <c r="Y337" s="4" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="Z337" s="4" t="s">
         <v>366</v>
       </c>
       <c r="AA337" s="4" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="AB337" s="20">
         <v>1.1348</v>
@@ -71001,7 +70984,7 @@
         <v>4</v>
       </c>
       <c r="N338" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O338" s="7">
         <v>22.4</v>
@@ -71033,13 +71016,13 @@
         <v>367</v>
       </c>
       <c r="Y338" s="4" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="Z338" s="4" t="s">
         <v>367</v>
       </c>
       <c r="AA338" s="4" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="AB338" s="20">
         <v>1.1024</v>
@@ -71110,7 +71093,7 @@
         <v>4</v>
       </c>
       <c r="N339" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O339" s="7">
         <v>28.8</v>
@@ -71142,13 +71125,13 @@
         <v>368</v>
       </c>
       <c r="Y339" s="4" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="Z339" s="4" t="s">
         <v>368</v>
       </c>
       <c r="AA339" s="4" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="AB339" s="20">
         <v>0.91090000000000004</v>
@@ -71219,7 +71202,7 @@
         <v>4</v>
       </c>
       <c r="N340" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O340" s="4">
         <v>32.299999999999997</v>
@@ -71359,7 +71342,7 @@
         <v>4</v>
       </c>
       <c r="N342" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O342" s="4">
         <v>29.1</v>
@@ -71569,7 +71552,7 @@
         <v>4</v>
       </c>
       <c r="N345" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O345" s="4">
         <v>29.8</v>
@@ -71639,7 +71622,7 @@
         <v>4</v>
       </c>
       <c r="N346" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O346" s="4">
         <v>17.8</v>
@@ -71709,7 +71692,7 @@
         <v>4</v>
       </c>
       <c r="N347" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O347" s="4">
         <v>27.7</v>
@@ -71779,7 +71762,7 @@
         <v>4</v>
       </c>
       <c r="N348" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O348" s="4">
         <v>19.100000000000001</v>
@@ -71849,7 +71832,7 @@
         <v>4</v>
       </c>
       <c r="N349" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O349" s="4">
         <v>33.5</v>
@@ -71919,7 +71902,7 @@
         <v>4</v>
       </c>
       <c r="N350" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O350" s="4">
         <v>29.6</v>
@@ -71989,7 +71972,7 @@
         <v>4</v>
       </c>
       <c r="N351" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O351" s="4">
         <v>27.1</v>
@@ -72059,7 +72042,7 @@
         <v>4</v>
       </c>
       <c r="N352" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O352" s="4">
         <v>26.5</v>
@@ -72129,7 +72112,7 @@
         <v>4</v>
       </c>
       <c r="N353" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O353" s="4">
         <v>23.1</v>
@@ -72199,7 +72182,7 @@
         <v>4</v>
       </c>
       <c r="N354" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O354" s="4">
         <v>28.8</v>
@@ -72339,7 +72322,7 @@
         <v>4</v>
       </c>
       <c r="N356" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O356" s="4">
         <v>28</v>
@@ -72409,7 +72392,7 @@
         <v>4</v>
       </c>
       <c r="N357" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O357" s="4">
         <v>30.9</v>
@@ -72549,7 +72532,7 @@
         <v>4</v>
       </c>
       <c r="N359" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O359" s="4">
         <v>25.4</v>
@@ -72619,7 +72602,7 @@
         <v>4</v>
       </c>
       <c r="N360" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O360" s="4">
         <v>27.6</v>
@@ -72829,7 +72812,7 @@
         <v>4</v>
       </c>
       <c r="N363" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O363" s="4">
         <v>31.3</v>
@@ -72899,7 +72882,7 @@
         <v>4</v>
       </c>
       <c r="N364" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O364" s="4">
         <v>25.7</v>
@@ -73109,7 +73092,7 @@
         <v>4</v>
       </c>
       <c r="N367" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O367" s="4">
         <v>29.2</v>
@@ -73249,7 +73232,7 @@
         <v>4</v>
       </c>
       <c r="N369" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O369" s="4">
         <v>17</v>
@@ -73389,7 +73372,7 @@
         <v>4</v>
       </c>
       <c r="N371" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O371" s="4">
         <v>31</v>
@@ -73459,7 +73442,7 @@
         <v>4</v>
       </c>
       <c r="N372" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O372" s="4">
         <v>27.1</v>
@@ -73529,7 +73512,7 @@
         <v>4</v>
       </c>
       <c r="N373" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O373" s="4">
         <v>24.3</v>
@@ -73669,7 +73652,7 @@
         <v>4</v>
       </c>
       <c r="N375" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O375" s="4">
         <v>24.3</v>
@@ -73739,7 +73722,7 @@
         <v>4</v>
       </c>
       <c r="N376" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O376" s="4">
         <v>29.5</v>
@@ -73809,7 +73792,7 @@
         <v>4</v>
       </c>
       <c r="N377" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O377" s="4">
         <v>26.8</v>
@@ -73879,7 +73862,7 @@
         <v>4</v>
       </c>
       <c r="N378" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O378" s="4">
         <v>14.3</v>
@@ -74019,7 +74002,7 @@
         <v>4</v>
       </c>
       <c r="N380" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O380" s="4">
         <v>16.399999999999999</v>
@@ -74089,7 +74072,7 @@
         <v>4</v>
       </c>
       <c r="N381" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O381" s="4">
         <v>27.6</v>
@@ -74159,7 +74142,7 @@
         <v>4</v>
       </c>
       <c r="N382" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O382" s="4">
         <v>31.3</v>
@@ -74229,7 +74212,7 @@
         <v>4</v>
       </c>
       <c r="N383" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O383" s="4">
         <v>29</v>
@@ -74299,7 +74282,7 @@
         <v>4</v>
       </c>
       <c r="N384" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O384" s="4">
         <v>29.5</v>
@@ -74369,7 +74352,7 @@
         <v>4</v>
       </c>
       <c r="N385" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O385" s="4">
         <v>24.5</v>
@@ -74439,7 +74422,7 @@
         <v>4</v>
       </c>
       <c r="N386" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O386" s="4">
         <v>26.3</v>
@@ -74509,7 +74492,7 @@
         <v>4</v>
       </c>
       <c r="N387" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O387" s="4">
         <v>25.3</v>
@@ -74579,7 +74562,7 @@
         <v>4</v>
       </c>
       <c r="N388" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O388" s="4">
         <v>26.2</v>
@@ -74649,7 +74632,7 @@
         <v>4</v>
       </c>
       <c r="N389" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O389" s="4">
         <v>23.5</v>
@@ -74719,7 +74702,7 @@
         <v>4</v>
       </c>
       <c r="N390" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O390" s="4">
         <v>28.8</v>
@@ -74789,7 +74772,7 @@
         <v>4</v>
       </c>
       <c r="N391" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O391" s="4">
         <v>28.4</v>
@@ -74859,7 +74842,7 @@
         <v>4</v>
       </c>
       <c r="N392" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O392" s="4">
         <v>22.9</v>
@@ -74999,7 +74982,7 @@
         <v>4</v>
       </c>
       <c r="N394" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O394" s="4">
         <v>28.8</v>
@@ -75069,7 +75052,7 @@
         <v>4</v>
       </c>
       <c r="N395" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O395" s="4">
         <v>30.5</v>
@@ -75139,7 +75122,7 @@
         <v>4</v>
       </c>
       <c r="N396" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O396" s="4">
         <v>27</v>
@@ -75209,7 +75192,7 @@
         <v>4</v>
       </c>
       <c r="N397" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O397" s="4">
         <v>23.8</v>
@@ -75279,7 +75262,7 @@
         <v>4</v>
       </c>
       <c r="N398" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O398" s="4">
         <v>21.4</v>
@@ -75349,7 +75332,7 @@
         <v>4</v>
       </c>
       <c r="N399" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O399" s="4">
         <v>22.5</v>
@@ -75419,7 +75402,7 @@
         <v>4</v>
       </c>
       <c r="N400" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O400" s="4">
         <v>20.8</v>
@@ -75489,7 +75472,7 @@
         <v>4</v>
       </c>
       <c r="N401" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O401" s="4">
         <v>20.5</v>
@@ -75559,7 +75542,7 @@
         <v>4</v>
       </c>
       <c r="N402" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O402" s="4">
         <v>20.2</v>
@@ -75629,7 +75612,7 @@
         <v>4</v>
       </c>
       <c r="N403" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O403" s="4">
         <v>26.1</v>
@@ -75699,7 +75682,7 @@
         <v>4</v>
       </c>
       <c r="N404" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O404" s="4">
         <v>28.2</v>
@@ -75769,7 +75752,7 @@
         <v>4</v>
       </c>
       <c r="N405" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O405" s="4">
         <v>21.9</v>
@@ -75839,7 +75822,7 @@
         <v>4</v>
       </c>
       <c r="N406" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O406" s="4">
         <v>29.3</v>
@@ -75909,7 +75892,7 @@
         <v>4</v>
       </c>
       <c r="N407" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O407" s="4">
         <v>18.100000000000001</v>
@@ -75979,7 +75962,7 @@
         <v>4</v>
       </c>
       <c r="N408" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O408" s="4">
         <v>17.399999999999999</v>
@@ -76049,7 +76032,7 @@
         <v>4</v>
       </c>
       <c r="N409" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O409" s="4">
         <v>15.2</v>
@@ -76080,7 +76063,7 @@
     </row>
     <row r="410" spans="1:50">
       <c r="A410" s="4" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B410" s="9" t="s">
         <v>472</v>
@@ -76145,16 +76128,16 @@
         <v>540</v>
       </c>
       <c r="W410" s="4" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="X410" s="4" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="Y410" s="4">
         <v>1</v>
       </c>
       <c r="Z410" s="4" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="AA410" s="4">
         <v>1</v>
@@ -76211,7 +76194,7 @@
     </row>
     <row r="411" spans="1:50">
       <c r="A411" s="4" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="B411" s="9" t="s">
         <v>472</v>
@@ -76276,16 +76259,16 @@
         <v>540</v>
       </c>
       <c r="W411" s="4" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="X411" s="4" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="Y411" s="4">
         <v>2</v>
       </c>
       <c r="Z411" s="4" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="AA411" s="4">
         <v>2</v>
@@ -76345,7 +76328,7 @@
     </row>
     <row r="412" spans="1:50">
       <c r="A412" s="4" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="B412" s="9" t="s">
         <v>472</v>
@@ -76384,7 +76367,7 @@
         <v>4</v>
       </c>
       <c r="N412" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O412" s="7">
         <v>30.2</v>
@@ -76410,16 +76393,16 @@
         <v>540</v>
       </c>
       <c r="W412" s="4" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="X412" s="4" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="Y412" s="4">
         <v>3</v>
       </c>
       <c r="Z412" s="4" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="AA412" s="4">
         <v>3</v>
@@ -76479,7 +76462,7 @@
     </row>
     <row r="413" spans="1:50">
       <c r="A413" s="4" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="B413" s="9" t="s">
         <v>472</v>
@@ -76518,7 +76501,7 @@
         <v>4</v>
       </c>
       <c r="N413" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O413" s="7">
         <v>34.1</v>
@@ -76544,16 +76527,16 @@
         <v>540</v>
       </c>
       <c r="W413" s="4" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="X413" s="4" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="Y413" s="4">
         <v>4</v>
       </c>
       <c r="Z413" s="4" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="AA413" s="4">
         <v>4</v>
@@ -76610,7 +76593,7 @@
     </row>
     <row r="414" spans="1:50">
       <c r="A414" s="4" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="B414" s="9" t="s">
         <v>472</v>
@@ -76675,16 +76658,16 @@
         <v>540</v>
       </c>
       <c r="W414" s="4" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="X414" s="4" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="Y414" s="4">
         <v>5</v>
       </c>
       <c r="Z414" s="4" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="AA414" s="4">
         <v>5</v>
@@ -76741,7 +76724,7 @@
     </row>
     <row r="415" spans="1:50">
       <c r="A415" s="4" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B415" s="9" t="s">
         <v>472</v>
@@ -76806,16 +76789,16 @@
         <v>540</v>
       </c>
       <c r="W415" s="4" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="X415" s="4" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="Y415" s="4">
         <v>6</v>
       </c>
       <c r="Z415" s="4" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="AA415" s="4">
         <v>6</v>
@@ -76875,7 +76858,7 @@
     </row>
     <row r="416" spans="1:50">
       <c r="A416" s="4" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="B416" s="9" t="s">
         <v>472</v>
@@ -76940,16 +76923,16 @@
         <v>540</v>
       </c>
       <c r="W416" s="4" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="X416" s="4" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="Y416" s="4">
         <v>7</v>
       </c>
       <c r="Z416" s="4" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="AA416" s="4">
         <v>7</v>
@@ -77006,7 +76989,7 @@
     </row>
     <row r="417" spans="1:50">
       <c r="A417" s="4" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="B417" s="9" t="s">
         <v>472</v>
@@ -77045,7 +77028,7 @@
         <v>4</v>
       </c>
       <c r="N417" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O417" s="7">
         <v>30.7</v>
@@ -77071,16 +77054,16 @@
         <v>540</v>
       </c>
       <c r="W417" s="4" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="X417" s="4" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="Y417" s="4">
         <v>8</v>
       </c>
       <c r="Z417" s="4" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="AA417" s="4">
         <v>8</v>
@@ -77137,7 +77120,7 @@
     </row>
     <row r="418" spans="1:50">
       <c r="A418" s="4" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="B418" s="9" t="s">
         <v>472</v>
@@ -77202,16 +77185,16 @@
         <v>540</v>
       </c>
       <c r="W418" s="4" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="X418" s="4" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="Y418" s="4">
         <v>9</v>
       </c>
       <c r="Z418" s="4" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="AA418" s="4">
         <v>9</v>
@@ -77244,34 +77227,13 @@
       <c r="AP418" s="4">
         <v>94.968553459999995</v>
       </c>
-      <c r="AQ418" s="4" t="s">
-        <v>555</v>
-      </c>
-      <c r="AR418" s="4" t="s">
-        <v>555</v>
-      </c>
-      <c r="AS418" s="4" t="s">
-        <v>555</v>
-      </c>
-      <c r="AT418" s="4" t="s">
-        <v>555</v>
-      </c>
-      <c r="AU418" s="4" t="s">
-        <v>555</v>
-      </c>
-      <c r="AV418" s="4" t="s">
-        <v>555</v>
-      </c>
-      <c r="AW418" s="4" t="s">
-        <v>555</v>
-      </c>
       <c r="AX418" s="27">
         <v>86</v>
       </c>
     </row>
     <row r="419" spans="1:50">
       <c r="A419" s="4" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="B419" s="9" t="s">
         <v>472</v>
@@ -77336,16 +77298,16 @@
         <v>540</v>
       </c>
       <c r="W419" s="4" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="X419" s="4" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="Y419" s="4">
         <v>10</v>
       </c>
       <c r="Z419" s="4" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="AA419" s="4">
         <v>10</v>
@@ -77405,7 +77367,7 @@
     </row>
     <row r="420" spans="1:50">
       <c r="A420" s="4" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="B420" s="9" t="s">
         <v>472</v>
@@ -77444,7 +77406,7 @@
         <v>4</v>
       </c>
       <c r="N420" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O420" s="7">
         <v>25.7</v>
@@ -77470,16 +77432,16 @@
         <v>540</v>
       </c>
       <c r="W420" s="4" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="X420" s="4" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="Y420" s="4">
         <v>11</v>
       </c>
       <c r="Z420" s="4" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="AA420" s="4">
         <v>11</v>
@@ -77515,7 +77477,7 @@
     </row>
     <row r="421" spans="1:50">
       <c r="A421" s="4" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="B421" s="9" t="s">
         <v>472</v>
@@ -77554,7 +77516,7 @@
         <v>4</v>
       </c>
       <c r="N421" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O421" s="7">
         <v>28.9</v>
@@ -77580,16 +77542,16 @@
         <v>540</v>
       </c>
       <c r="W421" s="4" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="X421" s="4" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="Y421" s="4">
         <v>12</v>
       </c>
       <c r="Z421" s="4" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="AA421" s="4">
         <v>12</v>
@@ -77625,7 +77587,7 @@
     </row>
     <row r="422" spans="1:50">
       <c r="A422" s="4" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="B422" s="17" t="s">
         <v>472</v>
@@ -77664,7 +77626,7 @@
         <v>4</v>
       </c>
       <c r="N422" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O422" s="4">
         <v>29.9</v>
@@ -77689,12 +77651,12 @@
         <v>533</v>
       </c>
       <c r="W422" s="4" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="423" spans="1:50">
       <c r="A423" s="4" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="B423" s="17" t="s">
         <v>472</v>
@@ -77733,7 +77695,7 @@
         <v>4</v>
       </c>
       <c r="N423" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O423" s="4">
         <v>29.3</v>
@@ -77758,12 +77720,12 @@
         <v>533</v>
       </c>
       <c r="W423" s="4" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="424" spans="1:50">
       <c r="A424" s="4" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="B424" s="17" t="s">
         <v>472</v>
@@ -77827,12 +77789,12 @@
         <v>533</v>
       </c>
       <c r="W424" s="4" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="425" spans="1:50">
       <c r="A425" s="4" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B425" s="17" t="s">
         <v>472</v>
@@ -77871,7 +77833,7 @@
         <v>4</v>
       </c>
       <c r="N425" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="O425" s="4">
         <v>25.8</v>
@@ -77896,7 +77858,7 @@
         <v>533</v>
       </c>
       <c r="W425" s="4" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="427" spans="1:50">
@@ -77931,156 +77893,156 @@
         <v>315</v>
       </c>
       <c r="F7" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="G7" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="H7" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="I7" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="8" spans="4:9" ht="12.75" customHeight="1">
       <c r="D8" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>466</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="G8" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="H8" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="I8" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="9" spans="4:9" ht="12.75" customHeight="1">
       <c r="D9" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>470</v>
       </c>
       <c r="H9" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="I9" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="10" spans="4:9" ht="12.75" customHeight="1">
       <c r="D10" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="E10">
         <v>2</v>
       </c>
       <c r="F10" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="G10" s="1" t="s">
+        <v>620</v>
+      </c>
+      <c r="H10" s="2" t="s">
         <v>621</v>
       </c>
-      <c r="H10" s="2" t="s">
-        <v>622</v>
-      </c>
       <c r="I10" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="11" spans="4:9" ht="12.75" customHeight="1">
       <c r="D11" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="E11">
         <v>3</v>
       </c>
       <c r="F11" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="G11" s="1" t="s">
+        <v>622</v>
+      </c>
+      <c r="H11" t="s">
         <v>623</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" s="2" t="s">
         <v>624</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>625</v>
       </c>
     </row>
     <row r="12" spans="4:9" ht="12.75" customHeight="1">
       <c r="D12" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="E12">
         <v>4</v>
       </c>
       <c r="F12" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="G12" s="1" t="s">
+        <v>625</v>
+      </c>
+      <c r="H12" t="s">
         <v>626</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" s="1" t="s">
         <v>627</v>
-      </c>
-      <c r="I12" s="1" t="s">
-        <v>628</v>
       </c>
     </row>
     <row r="13" spans="4:9" ht="12.75" customHeight="1">
       <c r="D13" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="E13">
         <v>5</v>
       </c>
       <c r="F13" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="G13" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="H13" t="s">
+        <v>628</v>
+      </c>
+      <c r="I13" s="1" t="s">
         <v>629</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>630</v>
       </c>
     </row>
     <row r="14" spans="4:9" ht="12.75" customHeight="1">
       <c r="D14" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="E14">
         <v>6</v>
       </c>
       <c r="F14" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="G14" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="H14" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
     </row>
     <row r="15" spans="4:9" ht="12.75" customHeight="1">
@@ -78092,7 +78054,7 @@
         <v>12</v>
       </c>
       <c r="F15" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="G15">
         <f>E15*3</f>
@@ -78209,22 +78171,22 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="B1" t="s">
+        <v>631</v>
+      </c>
+      <c r="C1" t="s">
         <v>632</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>633</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>634</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>635</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>636</v>
-      </c>
-      <c r="G1" t="s">
-        <v>637</v>
       </c>
     </row>
     <row r="2" spans="1:7">

</xml_diff>